<commit_message>
DOC(jdt) :jdt du 30.01.2026
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
+++ b/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\py13koy\Documents\GitHub\Dash-Project\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B61B89-BE35-4D66-9BC0-4DE98E57E9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71616FB1-B726-4134-A1E0-981D148E3380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="46">
   <si>
     <t>Auteur:</t>
   </si>
@@ -167,6 +167,18 @@
   </si>
   <si>
     <t>WIP</t>
+  </si>
+  <si>
+    <t>dust trail effect pour les mouvement du player</t>
+  </si>
+  <si>
+    <t>rotation du player quand il saute</t>
+  </si>
+  <si>
+    <t>fix les pariticule pour quelle soit toujours en bas du player</t>
+  </si>
+  <si>
+    <t>modification de 2 sprite (Speed 2/3)</t>
   </si>
 </sst>
 </file>
@@ -1109,7 +1121,7 @@
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>150</c:v>
+                  <c:v>295</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>15</c:v>
@@ -1958,13 +1970,13 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>8.3333333333333329E-2</c:v>
+                  <c:v>4.6153846153846156E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.83333333333333337</c:v>
+                  <c:v>0.90769230769230769</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.3333333333333329E-2</c:v>
+                  <c:v>4.6153846153846156E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4202,7 +4214,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 0 minutes</v>
+        <v>5 heures 25 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4217,15 +4229,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>180</v>
+        <v>265</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>180</v>
+        <v>325</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4527,72 +4539,112 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="74" t="str">
+      <c r="A17" s="74">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="40"/>
+        <v>5</v>
+      </c>
+      <c r="B17" s="40">
+        <v>46052</v>
+      </c>
       <c r="C17" s="41"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="28"/>
+      <c r="D17" s="42">
+        <v>35</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="28" t="s">
+        <v>40</v>
+      </c>
       <c r="G17" s="46"/>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="73" t="str">
+      <c r="A18" s="73">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="36"/>
+        <v>5</v>
+      </c>
+      <c r="B18" s="36">
+        <v>46052</v>
+      </c>
       <c r="C18" s="37"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="28"/>
+      <c r="D18" s="38">
+        <v>30</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>42</v>
+      </c>
       <c r="G18" s="45"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="74" t="str">
+      <c r="A19" s="74">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="40"/>
+        <v>5</v>
+      </c>
+      <c r="B19" s="40">
+        <v>46052</v>
+      </c>
       <c r="C19" s="41"/>
-      <c r="D19" s="42"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="28"/>
+      <c r="D19" s="42">
+        <v>15</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>43</v>
+      </c>
       <c r="G19" s="46"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="73" t="str">
+      <c r="A20" s="73">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="36"/>
+        <v>5</v>
+      </c>
+      <c r="B20" s="36">
+        <v>46052</v>
+      </c>
       <c r="C20" s="37"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="28"/>
+      <c r="D20" s="38">
+        <v>5</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>44</v>
+      </c>
       <c r="G20" s="45"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="74" t="str">
+      <c r="A21" s="74">
         <f>IF(ISBLANK(B21),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="41"/>
+        <v>5</v>
+      </c>
+      <c r="B21" s="40">
+        <v>46052</v>
+      </c>
+      <c r="C21" s="41">
+        <v>1</v>
+      </c>
       <c r="D21" s="42"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="28"/>
+      <c r="E21" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>45</v>
+      </c>
       <c r="G21" s="46"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -10878,7 +10930,7 @@
       </c>
       <c r="G6" s="47">
         <f>SUM(A6:B6)/$C$10</f>
-        <v>8.3333333333333329E-2</v>
+        <v>4.6153846153846156E-2</v>
       </c>
       <c r="L6" s="62" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10895,15 +10947,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>150</v>
+        <v>235</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>295</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10911,11 +10963,11 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>2 h 30 min</v>
+        <v>4 h 55 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
-        <v>0.83333333333333337</v>
+        <v>0.90769230769230769</v>
       </c>
       <c r="L7" s="64" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10952,7 +11004,7 @@
       </c>
       <c r="G8" s="47">
         <f t="shared" si="2"/>
-        <v>8.3333333333333329E-2</v>
+        <v>4.6153846153846156E-2</v>
       </c>
       <c r="L8" s="65" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11006,26 +11058,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>180</v>
+        <v>265</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>180</v>
+        <v>325</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 00 min</v>
+        <v>5 h 25 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>3.4090909090909088E-2</v>
+        <v>6.1553030303030304E-2</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11064,6 +11116,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11073,15 +11134,6 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11298,6 +11350,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11306,14 +11366,6 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Doc(jdt) : jdt du 06.02.2025
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
+++ b/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\py13koy\Documents\GitHub\Dash-Project\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71616FB1-B726-4134-A1E0-981D148E3380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BCB07D-6AAB-4B47-A907-19A4DA657194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="55">
   <si>
     <t>Auteur:</t>
   </si>
@@ -179,6 +179,33 @@
   </si>
   <si>
     <t>modification de 2 sprite (Speed 2/3)</t>
+  </si>
+  <si>
+    <t>ajoute des changements de vitesse</t>
+  </si>
+  <si>
+    <t>ajout de l'invertion de gravité</t>
+  </si>
+  <si>
+    <t>rotation du player quand il est en l'air</t>
+  </si>
+  <si>
+    <t>tournais quand il étais au sol</t>
+  </si>
+  <si>
+    <t>création du mode vertical</t>
+  </si>
+  <si>
+    <t>création des portail de changement de mode</t>
+  </si>
+  <si>
+    <t>reset des parametre quand il respawn</t>
+  </si>
+  <si>
+    <t>pouvoir jump quand gravity up avec le nouveaux code</t>
+  </si>
+  <si>
+    <t>ajout gravity up pour vertical</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1148,7 @@
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>295</c:v>
+                  <c:v>475</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>15</c:v>
@@ -1970,13 +1997,13 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>4.6153846153846156E-2</c:v>
+                  <c:v>2.9702970297029702E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.90769230769230769</c:v>
+                  <c:v>0.94059405940594054</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6153846153846156E-2</c:v>
+                  <c:v>2.9702970297029702E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4214,7 +4241,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>5 heures 25 minutes</v>
+        <v>8 heures 25 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4229,15 +4256,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>265</v>
+        <v>385</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>325</v>
+        <v>505</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4648,99 +4675,165 @@
       <c r="G21" s="46"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="73" t="str">
+      <c r="A22" s="73">
         <f>IF(ISBLANK(B22),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="36"/>
+        <v>6</v>
+      </c>
+      <c r="B22" s="36">
+        <v>46059</v>
+      </c>
       <c r="C22" s="37"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="28"/>
+      <c r="D22" s="38">
+        <v>15</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>46</v>
+      </c>
       <c r="G22" s="45"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="74" t="str">
+      <c r="A23" s="74">
         <f>IF(ISBLANK(B23),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="40"/>
+        <v>6</v>
+      </c>
+      <c r="B23" s="40">
+        <v>46059</v>
+      </c>
       <c r="C23" s="41"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="28"/>
+      <c r="D23" s="42">
+        <v>10</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="28" t="s">
+        <v>47</v>
+      </c>
       <c r="G23" s="46"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="73" t="str">
+      <c r="A24" s="73">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
+        <v>6</v>
+      </c>
+      <c r="B24" s="36">
+        <v>46059</v>
+      </c>
+      <c r="C24" s="37">
+        <v>1</v>
+      </c>
       <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="45"/>
+      <c r="E24" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="G24" s="45" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="74" t="str">
+      <c r="A25" s="74">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="40"/>
+        <v>6</v>
+      </c>
+      <c r="B25" s="40">
+        <v>46059</v>
+      </c>
       <c r="C25" s="41"/>
-      <c r="D25" s="42"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="28"/>
+      <c r="D25" s="42">
+        <v>30</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>50</v>
+      </c>
       <c r="G25" s="46"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="73" t="str">
+      <c r="A26" s="73">
         <f>IF(ISBLANK(B26),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="36"/>
+        <v>6</v>
+      </c>
+      <c r="B26" s="36">
+        <v>46059</v>
+      </c>
       <c r="C26" s="37"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="28"/>
+      <c r="D26" s="38">
+        <v>20</v>
+      </c>
+      <c r="E26" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="28" t="s">
+        <v>51</v>
+      </c>
       <c r="G26" s="45"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="74" t="str">
+      <c r="A27" s="74">
         <f>IF(ISBLANK(B27),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B27))</f>
-        <v/>
-      </c>
-      <c r="B27" s="40"/>
+        <v>6</v>
+      </c>
+      <c r="B27" s="40">
+        <v>46059</v>
+      </c>
       <c r="C27" s="41"/>
-      <c r="D27" s="42"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="28"/>
+      <c r="D27" s="42">
+        <v>5</v>
+      </c>
+      <c r="E27" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="28" t="s">
+        <v>52</v>
+      </c>
       <c r="G27" s="46"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="73" t="str">
+      <c r="A28" s="73">
         <f>IF(ISBLANK(B28),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B28))</f>
-        <v/>
-      </c>
-      <c r="B28" s="36"/>
+        <v>6</v>
+      </c>
+      <c r="B28" s="36">
+        <v>46059</v>
+      </c>
       <c r="C28" s="37"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="27"/>
+      <c r="D28" s="38">
+        <v>30</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>53</v>
+      </c>
       <c r="G28" s="45"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="74" t="str">
+      <c r="A29" s="74">
         <f>IF(ISBLANK(B29),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B29))</f>
-        <v/>
-      </c>
-      <c r="B29" s="40"/>
+        <v>6</v>
+      </c>
+      <c r="B29" s="40">
+        <v>46059</v>
+      </c>
       <c r="C29" s="41"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="27"/>
+      <c r="D29" s="42">
+        <v>10</v>
+      </c>
+      <c r="E29" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>54</v>
+      </c>
       <c r="G29" s="46"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -10930,7 +11023,7 @@
       </c>
       <c r="G6" s="47">
         <f>SUM(A6:B6)/$C$10</f>
-        <v>4.6153846153846156E-2</v>
+        <v>2.9702970297029702E-2</v>
       </c>
       <c r="L6" s="62" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10947,15 +11040,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>235</v>
+        <v>355</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>295</v>
+        <v>475</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10963,11 +11056,11 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>4 h 55 min</v>
+        <v>7 h 55 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
-        <v>0.90769230769230769</v>
+        <v>0.94059405940594054</v>
       </c>
       <c r="L7" s="64" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11004,7 +11097,7 @@
       </c>
       <c r="G8" s="47">
         <f t="shared" si="2"/>
-        <v>4.6153846153846156E-2</v>
+        <v>2.9702970297029702E-2</v>
       </c>
       <c r="L8" s="65" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11058,26 +11151,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>265</v>
+        <v>385</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>325</v>
+        <v>505</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>5 h 25 min</v>
+        <v>8 h 25 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>6.1553030303030304E-2</v>
+        <v>9.5643939393939392E-2</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11116,15 +11209,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11134,6 +11218,15 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11350,14 +11443,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11366,6 +11451,14 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Doc(jdt) jdt du 13.02.2026
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
+++ b/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\py13koy\Documents\GitHub\Dash-Project\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BCB07D-6AAB-4B47-A907-19A4DA657194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8DF392-ED1A-43D4-8AB0-26EF4609780C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
   <si>
     <t>Auteur:</t>
   </si>
@@ -206,6 +206,21 @@
   </si>
   <si>
     <t>ajout gravity up pour vertical</t>
+  </si>
+  <si>
+    <t>ajout des mirror portal (invertion du sense)</t>
+  </si>
+  <si>
+    <t>j'ai du modifier les boost de speed pour qu'il garde le meme sense de vitesse</t>
+  </si>
+  <si>
+    <t>ajout du bump (force le saut)</t>
+  </si>
+  <si>
+    <t>modification du code de saut pour qu'il saute la meme distance peu importe la vitesse</t>
+  </si>
+  <si>
+    <t>réglé le prolème de saut (ne saute pas tout le temps)</t>
   </si>
 </sst>
 </file>
@@ -1148,7 +1163,7 @@
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>475</c:v>
+                  <c:v>660</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>15</c:v>
@@ -1997,13 +2012,13 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2.9702970297029702E-2</c:v>
+                  <c:v>2.1739130434782608E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.94059405940594054</c:v>
+                  <c:v>0.95652173913043481</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.9702970297029702E-2</c:v>
+                  <c:v>2.1739130434782608E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4241,7 +4256,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>8 heures 25 minutes</v>
+        <v>11 heures 30 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4256,15 +4271,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>385</v>
+        <v>510</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>505</v>
+        <v>690</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4837,64 +4852,112 @@
       <c r="G29" s="46"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="73" t="str">
+      <c r="A30" s="73">
         <f>IF(ISBLANK(B30),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B30))</f>
-        <v/>
-      </c>
-      <c r="B30" s="36"/>
+        <v>7</v>
+      </c>
+      <c r="B30" s="36">
+        <v>46066</v>
+      </c>
       <c r="C30" s="37"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="28"/>
-      <c r="G30" s="45"/>
+      <c r="D30" s="38">
+        <v>40</v>
+      </c>
+      <c r="E30" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="G30" s="45" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="74" t="str">
+      <c r="A31" s="74">
         <f>IF(ISBLANK(B31),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B31))</f>
-        <v/>
-      </c>
-      <c r="B31" s="40"/>
+        <v>7</v>
+      </c>
+      <c r="B31" s="40">
+        <v>46066</v>
+      </c>
       <c r="C31" s="41"/>
-      <c r="D31" s="42"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="27"/>
+      <c r="D31" s="42">
+        <v>15</v>
+      </c>
+      <c r="E31" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>57</v>
+      </c>
       <c r="G31" s="46"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="73" t="str">
+      <c r="A32" s="73">
         <f>IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
-        <v/>
-      </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="37"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="45"/>
+        <v>7</v>
+      </c>
+      <c r="B32" s="36">
+        <v>46066</v>
+      </c>
+      <c r="C32" s="37">
+        <v>1</v>
+      </c>
+      <c r="D32" s="38">
+        <v>40</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F32" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="G32" s="45" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="74" t="str">
+      <c r="A33" s="74">
         <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
-        <v/>
-      </c>
-      <c r="B33" s="40"/>
+        <v>7</v>
+      </c>
+      <c r="B33" s="40">
+        <v>46066</v>
+      </c>
       <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="27"/>
+      <c r="D33" s="42">
+        <v>25</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>59</v>
+      </c>
       <c r="G33" s="46"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="73" t="str">
+      <c r="A34" s="73">
         <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="36"/>
+        <v>7</v>
+      </c>
+      <c r="B34" s="36">
+        <v>46066</v>
+      </c>
       <c r="C34" s="37"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="39"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="45"/>
+      <c r="D34" s="38">
+        <v>5</v>
+      </c>
+      <c r="E34" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F34" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="G34" s="45" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="74" t="str">
@@ -11023,7 +11086,7 @@
       </c>
       <c r="G6" s="47">
         <f>SUM(A6:B6)/$C$10</f>
-        <v>2.9702970297029702E-2</v>
+        <v>2.1739130434782608E-2</v>
       </c>
       <c r="L6" s="62" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11040,15 +11103,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>355</v>
+        <v>480</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>475</v>
+        <v>660</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11056,11 +11119,11 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>7 h 55 min</v>
+        <v>11 h 00 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
-        <v>0.94059405940594054</v>
+        <v>0.95652173913043481</v>
       </c>
       <c r="L7" s="64" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11097,7 +11160,7 @@
       </c>
       <c r="G8" s="47">
         <f t="shared" si="2"/>
-        <v>2.9702970297029702E-2</v>
+        <v>2.1739130434782608E-2</v>
       </c>
       <c r="L8" s="65" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11151,26 +11214,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>385</v>
+        <v>510</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>505</v>
+        <v>690</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>8 h 25 min</v>
+        <v>11 h 30 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>9.5643939393939392E-2</v>
+        <v>0.13068181818181818</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11209,6 +11272,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11218,15 +11290,6 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11443,6 +11506,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11451,14 +11522,6 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Feat(JDT) : jdt du 27.02.2026
[DONE]
jdt pendant les cours
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
+++ b/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\py13koy\Documents\GitHub\Dash-Project\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8DF392-ED1A-43D4-8AB0-26EF4609780C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714A4D4C-2D13-47DD-A0E9-2581D3D2E531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="65">
   <si>
     <t>Auteur:</t>
   </si>
@@ -221,6 +221,21 @@
   </si>
   <si>
     <t>réglé le prolème de saut (ne saute pas tout le temps)</t>
+  </si>
+  <si>
+    <t>j'ai voulu faire tout avec 1 seul GroundCheck (sa bug tout)</t>
+  </si>
+  <si>
+    <t>modification du code de saut pour qu'il saute la meme distance peu importe la vitesse mode normal</t>
+  </si>
+  <si>
+    <t>modification du code de saut pour qu'il saute la meme distance peu importe la vitesse mode GravityUp</t>
+  </si>
+  <si>
+    <t>modification du code de saut pour qu'il saute la meme distance peu importe la vitesse mode vertical</t>
+  </si>
+  <si>
+    <t>Rapport</t>
   </si>
 </sst>
 </file>
@@ -1163,13 +1178,13 @@
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>660</c:v>
+                  <c:v>795</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2012,16 +2027,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>2.1739130434782608E-2</c:v>
+                  <c:v>1.7241379310344827E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.95652173913043481</c:v>
+                  <c:v>0.91379310344827591</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.1739130434782608E-2</c:v>
+                  <c:v>1.7241379310344827E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>5.1724137931034482E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4256,7 +4271,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>11 heures 30 minutes</v>
+        <v>14 heures 30 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4271,15 +4286,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>510</v>
+        <v>630</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>690</v>
+        <v>870</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4959,52 +4974,88 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="74" t="str">
+    <row r="35" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="74">
         <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="40"/>
+        <v>9</v>
+      </c>
+      <c r="B35" s="40">
+        <v>46080</v>
+      </c>
       <c r="C35" s="41"/>
-      <c r="D35" s="42"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="28"/>
+      <c r="D35" s="42">
+        <v>25</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" s="28" t="s">
+        <v>61</v>
+      </c>
       <c r="G35" s="46"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="73" t="str">
+      <c r="A36" s="73">
         <f>IF(ISBLANK(B36),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B36))</f>
-        <v/>
-      </c>
-      <c r="B36" s="36"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="45"/>
+        <v>9</v>
+      </c>
+      <c r="B36" s="36">
+        <v>46080</v>
+      </c>
+      <c r="C36" s="37">
+        <v>1</v>
+      </c>
+      <c r="D36" s="38">
+        <v>25</v>
+      </c>
+      <c r="E36" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" s="27" t="s">
+        <v>62</v>
+      </c>
+      <c r="G36" s="45" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="74" t="str">
+      <c r="A37" s="74">
         <f>IF(ISBLANK(B37),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B37))</f>
-        <v/>
-      </c>
-      <c r="B37" s="40"/>
+        <v>9</v>
+      </c>
+      <c r="B37" s="40">
+        <v>46080</v>
+      </c>
       <c r="C37" s="41"/>
-      <c r="D37" s="42"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="27"/>
+      <c r="D37" s="42">
+        <v>25</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="F37" s="27" t="s">
+        <v>63</v>
+      </c>
       <c r="G37" s="46"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="73" t="str">
+      <c r="A38" s="73">
         <f>IF(ISBLANK(B38),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B38))</f>
-        <v/>
-      </c>
-      <c r="B38" s="36"/>
+        <v>9</v>
+      </c>
+      <c r="B38" s="36">
+        <v>46080</v>
+      </c>
       <c r="C38" s="37"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="39"/>
-      <c r="F38" s="27"/>
+      <c r="D38" s="38">
+        <v>45</v>
+      </c>
+      <c r="E38" s="39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F38" s="27" t="s">
+        <v>64</v>
+      </c>
       <c r="G38" s="45"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -11086,7 +11137,7 @@
       </c>
       <c r="G6" s="47">
         <f>SUM(A6:B6)/$C$10</f>
-        <v>2.1739130434782608E-2</v>
+        <v>1.7241379310344827E-2</v>
       </c>
       <c r="L6" s="62" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11103,15 +11154,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>480</v>
+        <v>555</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>660</v>
+        <v>795</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11119,11 +11170,11 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>11 h 00 min</v>
+        <v>13 h 15 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
-        <v>0.95652173913043481</v>
+        <v>0.91379310344827591</v>
       </c>
       <c r="L7" s="64" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11160,7 +11211,7 @@
       </c>
       <c r="G8" s="47">
         <f t="shared" si="2"/>
-        <v>2.1739130434782608E-2</v>
+        <v>1.7241379310344827E-2</v>
       </c>
       <c r="L8" s="65" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11181,11 +11232,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E9" s="23" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11193,11 +11244,11 @@
       </c>
       <c r="F9" s="55" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>0 h 45 min</v>
       </c>
       <c r="G9" s="56">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.1724137931034482E-2</v>
       </c>
       <c r="L9" s="66" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11214,26 +11265,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>510</v>
+        <v>630</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>690</v>
+        <v>870</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>11 h 30 min</v>
+        <v>14 h 30 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.13068181818181818</v>
+        <v>0.16477272727272727</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11272,15 +11323,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11290,6 +11332,15 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11506,14 +11557,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11522,6 +11565,14 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Doc(jdt) jdt du 06.03.2026
</commit_message>
<xml_diff>
--- a/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
+++ b/Doc/Journal-de-Travail_RubertiGianmarco.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\py13koy\Documents\GitHub\Dash-Project\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714A4D4C-2D13-47DD-A0E9-2581D3D2E531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CACA8380-14BA-48CA-B4EA-F57D0D317688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="66">
   <si>
     <t>Auteur:</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Rapport</t>
+  </si>
+  <si>
+    <t>amélioration de la gestion de la caméra</t>
   </si>
 </sst>
 </file>
@@ -1178,13 +1181,13 @@
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>795</c:v>
+                  <c:v>860</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45</c:v>
+                  <c:v>105</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2027,16 +2030,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.7241379310344827E-2</c:v>
+                  <c:v>1.507537688442211E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.91379310344827591</c:v>
+                  <c:v>0.86432160804020097</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.7241379310344827E-2</c:v>
+                  <c:v>1.507537688442211E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.1724137931034482E-2</c:v>
+                  <c:v>0.10552763819095477</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4271,7 +4274,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>14 heures 30 minutes</v>
+        <v>16 heures 35 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4286,15 +4289,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>630</v>
+        <v>695</v>
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>870</v>
+        <v>995</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -5056,42 +5059,70 @@
       <c r="F38" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="G38" s="45"/>
+      <c r="G38" s="45" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="74" t="str">
+      <c r="A39" s="74">
         <f>IF(ISBLANK(B39),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B39))</f>
-        <v/>
-      </c>
-      <c r="B39" s="40"/>
+        <v>10</v>
+      </c>
+      <c r="B39" s="40">
+        <v>46087</v>
+      </c>
       <c r="C39" s="41"/>
-      <c r="D39" s="42"/>
-      <c r="E39" s="43"/>
-      <c r="F39" s="27"/>
+      <c r="D39" s="42">
+        <v>40</v>
+      </c>
+      <c r="E39" s="43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" s="27" t="s">
+        <v>64</v>
+      </c>
       <c r="G39" s="46"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="73" t="str">
+      <c r="A40" s="73">
         <f>IF(ISBLANK(B40),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B40))</f>
-        <v/>
-      </c>
-      <c r="B40" s="36"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="27"/>
+        <v>10</v>
+      </c>
+      <c r="B40" s="36">
+        <v>46087</v>
+      </c>
+      <c r="C40" s="37">
+        <v>1</v>
+      </c>
+      <c r="D40" s="38">
+        <v>5</v>
+      </c>
+      <c r="E40" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F40" s="27" t="s">
+        <v>65</v>
+      </c>
       <c r="G40" s="45"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="74" t="str">
+      <c r="A41" s="74">
         <f>IF(ISBLANK(B41),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B41))</f>
-        <v/>
-      </c>
-      <c r="B41" s="40"/>
+        <v>10</v>
+      </c>
+      <c r="B41" s="40">
+        <v>46087</v>
+      </c>
       <c r="C41" s="41"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="27"/>
+      <c r="D41" s="42">
+        <v>20</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F41" s="27" t="s">
+        <v>64</v>
+      </c>
       <c r="G41" s="46"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -11137,7 +11168,7 @@
       </c>
       <c r="G6" s="47">
         <f>SUM(A6:B6)/$C$10</f>
-        <v>1.7241379310344827E-2</v>
+        <v>1.507537688442211E-2</v>
       </c>
       <c r="L6" s="62" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11154,15 +11185,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>795</v>
+        <v>860</v>
       </c>
       <c r="E7" s="30" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11170,11 +11201,11 @@
       </c>
       <c r="F7" s="55" t="str">
         <f t="shared" ref="F7:F10" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>13 h 15 min</v>
+        <v>14 h 20 min</v>
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
-        <v>0.91379310344827591</v>
+        <v>0.86432160804020097</v>
       </c>
       <c r="L7" s="64" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11211,7 +11242,7 @@
       </c>
       <c r="G8" s="47">
         <f t="shared" si="2"/>
-        <v>1.7241379310344827E-2</v>
+        <v>1.507537688442211E-2</v>
       </c>
       <c r="L8" s="65" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11232,11 +11263,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>105</v>
       </c>
       <c r="E9" s="23" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11244,11 +11275,11 @@
       </c>
       <c r="F9" s="55" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 45 min</v>
+        <v>1 h 45 min</v>
       </c>
       <c r="G9" s="56">
         <f t="shared" si="2"/>
-        <v>5.1724137931034482E-2</v>
+        <v>0.10552763819095477</v>
       </c>
       <c r="L9" s="66" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11265,26 +11296,26 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
-        <v>630</v>
+        <v>695</v>
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>870</v>
+        <v>995</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>14 h 30 min</v>
+        <v>16 h 35 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.16477272727272727</v>
+        <v>0.1884469696969697</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11323,6 +11354,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11332,15 +11372,6 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11557,6 +11588,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11565,14 +11604,6 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>